<commit_message>
refactor(excel): simplify parseExcel API to accept PoInfo instead of PoConfig and poName
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/TestEntity.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/TestEntity.xlsx
@@ -487,14 +487,24 @@
           <t>1001</t>
         </is>
       </c>
-      <c r="B4" s="1"/>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>张三</t>
+        </is>
+      </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>男</t>
         </is>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="D4" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>PDM</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat(excel): support JSON array format for excelHeader parsing
Allow excelHeader to be specified as a JSON array string (e.g., `["基本信息","个人资料","姓名"]`)
in addition to the existing slash-delimited format. This enables headers containing the `/`
character to be properly parsed without ambiguity. Update test fixtures to use the new format
and adjust test entity configuration with new roleLevel field and updated age max constraint.
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/TestEntity.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/TestEntity.xlsx
@@ -429,10 +429,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>唯一标识</t>
@@ -446,8 +446,9 @@
       <c r="C1" s="0"/>
       <c r="D1" s="0"/>
       <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="0"/>
       <c r="B2" s="0" t="inlineStr">
         <is>
@@ -461,8 +462,13 @@
           <t>所属部门</t>
         </is>
       </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>角色/等级</t>
+        </is>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="0"/>
       <c r="B3" s="0" t="inlineStr">
         <is>
@@ -480,8 +486,9 @@
         </is>
       </c>
       <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>1001</t>
@@ -505,13 +512,15 @@
           <t>PDM</t>
         </is>
       </c>
+      <c r="F4" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B1:F1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576" showDropDown="0">

</xml_diff>